<commit_message>
wijzig pisolieten van PT naar PS
</commit_message>
<xml_diff>
--- a/src/main/resources/be/vlaanderen/bodemenondergrond/data/id/conceptscheme/sedimentairestructuurtype/sedimentairestructuurtype.xlsx
+++ b/src/main/resources/be/vlaanderen/bodemenondergrond/data/id/conceptscheme/sedimentairestructuurtype/sedimentairestructuurtype.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I65"/>
+  <dimension ref="A1:J64"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,1886 +407,2049 @@
         <v>type</v>
       </c>
       <c r="C1" t="str">
+        <v>dc\.identifier</v>
+      </c>
+      <c r="D1" t="str">
+        <v>definition</v>
+      </c>
+      <c r="E1" t="str">
         <v>inScheme</v>
-      </c>
-      <c r="D1" t="str">
-        <v>member</v>
-      </c>
-      <c r="E1" t="str">
-        <v>prefLabel</v>
       </c>
       <c r="F1" t="str">
         <v>notation</v>
       </c>
       <c r="G1" t="str">
+        <v>note</v>
+      </c>
+      <c r="H1" t="str">
+        <v>prefLabel</v>
+      </c>
+      <c r="I1" t="str">
         <v>topConceptOf</v>
       </c>
-      <c r="H1" t="str">
-        <v>dc\.identifier</v>
-      </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>hasTopConcept</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/collection/sedimentairestructuurtype/sedimentairestructuurtype</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/be</v>
       </c>
       <c r="B2" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#Collection</v>
+        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C2" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.be</v>
       </c>
       <c r="D2" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/0|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/10|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/11|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/12|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/13|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/14|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/15|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/16|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/17|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/18|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/19|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/1|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/20|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/21|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/22|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/23|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/24|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/25|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/26|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/27|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/28|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/29|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/2|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/30|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/31|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/32|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/33|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/34|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/35|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/36|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/37|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/38|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/3|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/40|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/41|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/42|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/43|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/44|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/45|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/46|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/47|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/48|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/49|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/4|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/50|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/51|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/52|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/53|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/54|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/55|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/56|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/57|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/58|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/59|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/5|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/60|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/61|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/62|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/6|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/7|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/8|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/9</v>
+        <v>Fenestrae. Holten van millimetergrootte in sedimentaire gesteente die geheel of gedeeltelijk opgevuld kunnen zijn door sediment of cement, gevormd door uitdroging of insluiting van lucht.</v>
       </c>
       <c r="E2" t="str">
-        <v>Collectie van sedimentairestructuurtype.</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F2" t="str">
-        <v>null</v>
+        <v>BE</v>
       </c>
       <c r="G2" t="str">
-        <v>null</v>
+        <v>Fenestrae. Holten van millimetergrootte in sedimentaire gesteente die geheel of gedeeltelijk opgevuld kunnen zijn door sediment of cement, gevormd door uitdroging of insluiting van lucht.</v>
       </c>
       <c r="H2" t="str">
-        <v>null</v>
+        <v>birdseyes</v>
       </c>
       <c r="I2" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J2" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/0</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/bk</v>
       </c>
       <c r="B3" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C3" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.bk</v>
       </c>
       <c r="D3" t="str">
-        <v>null</v>
+        <v>Korrels die bestaan uit de overblijfselen van organismen, vaak microscopische kalkskeletjes.</v>
       </c>
       <c r="E3" t="str">
-        <v>onbepaald</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F3" t="str">
-        <v>0</v>
+        <v>BK</v>
       </c>
       <c r="G3" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Korrels die bestaan uit de overblijfselen van organismen, vaak microscopische kalkskeletjes.</v>
       </c>
       <c r="H3" t="str">
-        <v>null</v>
+        <v>bioklasten</v>
       </c>
       <c r="I3" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J3" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/1</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/bo</v>
       </c>
       <c r="B4" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C4" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.bo</v>
       </c>
       <c r="D4" t="str">
-        <v>null</v>
+        <v>Kalksteen waarbij de korrels aaneengekit zijn door organismen.</v>
       </c>
       <c r="E4" t="str">
-        <v>straticulaties</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F4" t="str">
-        <v>1</v>
+        <v>BO</v>
       </c>
       <c r="G4" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Kalksteen waarbij de korrels aaneengekit zijn door organismen.</v>
       </c>
       <c r="H4" t="str">
-        <v>null</v>
+        <v>boundstone textuur</v>
       </c>
       <c r="I4" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J4" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/10</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/br</v>
       </c>
       <c r="B5" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C5" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.br</v>
       </c>
       <c r="D5" t="str">
-        <v>null</v>
+        <v>Klastisch met grove hoekige fragmenten.</v>
       </c>
       <c r="E5" t="str">
-        <v>slumping</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F5" t="str">
-        <v>10</v>
+        <v>BR</v>
       </c>
       <c r="G5" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Klastisch met grove hoekige fragmenten.</v>
       </c>
       <c r="H5" t="str">
-        <v>null</v>
+        <v>breccieus</v>
       </c>
       <c r="I5" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J5" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/11</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/bt</v>
       </c>
       <c r="B6" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C6" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.bt</v>
       </c>
       <c r="D6" t="str">
-        <v>null</v>
+        <v>Het omwoelen van sediment, hoofdzakelijk door gravende organismen.</v>
       </c>
       <c r="E6" t="str">
-        <v>compactiebreuken</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F6" t="str">
-        <v>11</v>
+        <v>BT</v>
       </c>
       <c r="G6" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Het omwoelen van sediment, hoofdzakelijk door gravende organismen.</v>
       </c>
       <c r="H6" t="str">
-        <v>null</v>
+        <v>bioturbatie</v>
       </c>
       <c r="I6" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J6" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/12</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/ca</v>
       </c>
       <c r="B7" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C7" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.ca</v>
       </c>
       <c r="D7" t="str">
-        <v>null</v>
+        <v>Een poederig, nodulair tot sterk verhard materiaal dat nabij het oppervlak gevormd is in een ariede tot semi-ariede omgeving, door cementatie door calciet, aangevoerd door grondwater in het sediment en de bodem.</v>
       </c>
       <c r="E7" t="str">
-        <v>'regendruppels' (cf. Planolites)</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F7" t="str">
-        <v>12</v>
+        <v>CA</v>
       </c>
       <c r="G7" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Een poederig, nodulair tot sterk verhard materiaal dat nabij het oppervlak gevormd is in een ariede tot semi-ariede omgeving, door cementatie door calciet, aangevoerd door grondwater in het sediment en de bodem.</v>
       </c>
       <c r="H7" t="str">
-        <v>null</v>
+        <v>calcrete / caliche</v>
       </c>
       <c r="I7" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J7" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/13</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/cb</v>
       </c>
       <c r="B8" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C8" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.cb</v>
       </c>
       <c r="D8" t="str">
-        <v>null</v>
+        <v>Breuken ontstaan door compactie van het sediment bij begraving.</v>
       </c>
       <c r="E8" t="str">
-        <v>erosievlak</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F8" t="str">
-        <v>13</v>
+        <v>CB</v>
       </c>
       <c r="G8" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Breuken ontstaan door compactie van het sediment bij begraving.</v>
       </c>
       <c r="H8" t="str">
-        <v>null</v>
+        <v>compactiebreuken</v>
       </c>
       <c r="I8" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J8" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/14</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/co</v>
       </c>
       <c r="B9" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C9" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.co</v>
       </c>
       <c r="D9" t="str">
-        <v>null</v>
+        <v>Nodule, vaak sferisch maar kan ook irregulair van vorm zijn. Vaak bestaande uit carbonaatmateriaal, pyriet, gips of silica.</v>
       </c>
       <c r="E9" t="str">
-        <v>niet-gecompacteerde fossielen</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F9" t="str">
-        <v>14</v>
+        <v>CO</v>
       </c>
       <c r="G9" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Nodule, vaak sferisch maar kan ook irregulair van vorm zijn. Vaak bestaande uit carbonaatmateriaal, pyriet, gips of silica.</v>
       </c>
       <c r="H9" t="str">
-        <v>null</v>
+        <v>concretie</v>
       </c>
       <c r="I9" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J9" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/15</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/cu</v>
       </c>
       <c r="B10" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C10" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.cu</v>
       </c>
       <c r="D10" t="str">
-        <v>null</v>
+        <v>Gelaagd sediment waarbij de korrelgrootte toeneemt naar boven toe.</v>
       </c>
       <c r="E10" t="str">
-        <v>micarijk vlak</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F10" t="str">
-        <v>15</v>
+        <v>CU</v>
       </c>
       <c r="G10" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Gelaagd sediment waarbij de korrelgrootte toeneemt naar boven toe.</v>
       </c>
       <c r="H10" t="str">
-        <v>null</v>
+        <v>CU-gegradeerde gelaagdheid</v>
       </c>
       <c r="I10" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J10" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/16</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/ep</v>
       </c>
       <c r="B11" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C11" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.ep</v>
       </c>
       <c r="D11" t="str">
-        <v>null</v>
+        <v>Een secundair evaporiet mineraal dat de vorm van het oorspronkelijke mineraal of fossiel heeft behouden.</v>
       </c>
       <c r="E11" t="str">
-        <v>zwart / kolig laagvlak</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F11" t="str">
-        <v>16</v>
+        <v>EP</v>
       </c>
       <c r="G11" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Een secundair evaporiet mineraal dat de vorm van het oorspronkelijke mineraal of fossiel heeft behouden.</v>
       </c>
       <c r="H11" t="str">
-        <v>null</v>
+        <v>evaporiet pseudomorfen</v>
       </c>
       <c r="I11" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J11" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/17</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/ev</v>
       </c>
       <c r="B12" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C12" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.ev</v>
       </c>
       <c r="D12" t="str">
-        <v>null</v>
+        <v>Een vlak (of lijn in een 2D profiel) waarop erosie heeft plaatsgevonden. Het bovenliggende pakket is ingesneden in het onderliggende pakket. Dit vlak kan recht of onregelmatig ondulerend zijn. Vaak is er een basisgrind aanwezig aan de basis van het bovenliggende pakket.</v>
       </c>
       <c r="E12" t="str">
-        <v>laagvlak met koolbrokjes</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F12" t="str">
-        <v>17</v>
+        <v>EV</v>
       </c>
       <c r="G12" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Een vlak (of lijn in een 2D profiel) waarop erosie heeft plaatsgevonden. Het bovenliggende pakket is ingesneden in het onderliggende pakket. Dit vlak kan recht of onregelmatig ondulerend zijn. Vaak is er een basisgrind aanwezig aan de basis van het bovenliggende pakket.</v>
       </c>
       <c r="H12" t="str">
-        <v>null</v>
+        <v>erosievlak</v>
       </c>
       <c r="I12" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J12" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/18</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/fb</v>
       </c>
       <c r="B13" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C13" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.fb</v>
       </c>
       <c r="D13" t="str">
-        <v>null</v>
+        <v>Aanwezigheid van fijne banken.</v>
       </c>
       <c r="E13" t="str">
-        <v>aangespoelde plantenresten / plantenhaksel</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F13" t="str">
-        <v>18</v>
+        <v>FB</v>
       </c>
       <c r="G13" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Aanwezigheid van fijne banken.</v>
       </c>
       <c r="H13" t="str">
-        <v>null</v>
+        <v>fijn gebankt</v>
       </c>
       <c r="I13" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J13" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/19</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/fn</v>
       </c>
       <c r="B14" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C14" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.fn</v>
       </c>
       <c r="D14" t="str">
-        <v>null</v>
+        <v>Fossiele die niet volledig gecompacteerd zijn tot platte afdrukken.</v>
       </c>
       <c r="E14" t="str">
-        <v>bioturbatie</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F14" t="str">
-        <v>19</v>
+        <v>FN</v>
       </c>
       <c r="G14" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Fossiele die niet volledig gecompacteerd zijn tot platte afdrukken.</v>
       </c>
       <c r="H14" t="str">
-        <v>null</v>
+        <v>niet-gecompacteerde fossielen</v>
       </c>
       <c r="I14" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J14" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/2</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/fo</v>
       </c>
       <c r="B15" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C15" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.fo</v>
       </c>
       <c r="D15" t="str">
-        <v>null</v>
+        <v>Sediment rijk aan fossielen.</v>
       </c>
       <c r="E15" t="str">
-        <v>laminaties</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F15" t="str">
-        <v>2</v>
+        <v>FO</v>
       </c>
       <c r="G15" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Sediment rijk aan fossielen.</v>
       </c>
       <c r="H15" t="str">
-        <v>null</v>
+        <v>fossielrijk</v>
       </c>
       <c r="I15" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J15" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/20</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/fs</v>
       </c>
       <c r="B16" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C16" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.fs</v>
       </c>
       <c r="D16" t="str">
-        <v>null</v>
+        <v>Een grofkorrelige kalksteen waarbij meer dan 10% van de klasten groter is dan 2 mm. De klasten worden door de matrix gedragen.</v>
       </c>
       <c r="E16" t="str">
-        <v>verspreide keien</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F16" t="str">
-        <v>20</v>
+        <v>FS</v>
       </c>
       <c r="G16" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Een grofkorrelige kalksteen waarbij meer dan 10% van de klasten groter is dan 2 mm. De klasten worden door de matrix gedragen.</v>
       </c>
       <c r="H16" t="str">
-        <v>null</v>
+        <v>floatstone</v>
       </c>
       <c r="I16" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J16" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/21</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/fu</v>
       </c>
       <c r="B17" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C17" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.fu</v>
       </c>
       <c r="D17" t="str">
-        <v>null</v>
+        <v>Gelaagd sediment waarbij de korrelgrootte afneemt naar boven toe.</v>
       </c>
       <c r="E17" t="str">
-        <v>mudstone textuur</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F17" t="str">
-        <v>21</v>
+        <v>FU</v>
       </c>
       <c r="G17" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Gelaagd sediment waarbij de korrelgrootte afneemt naar boven toe.</v>
       </c>
       <c r="H17" t="str">
-        <v>null</v>
+        <v>FU-gegradeerde gelaagdheid</v>
       </c>
       <c r="I17" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J17" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/22</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/ge</v>
       </c>
       <c r="B18" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C18" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.ge</v>
       </c>
       <c r="D18" t="str">
-        <v>null</v>
+        <v>Aanwezigheid van een gebande textuur.</v>
       </c>
       <c r="E18" t="str">
-        <v>wackestone textuur</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F18" t="str">
-        <v>22</v>
+        <v>GE</v>
       </c>
       <c r="G18" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Aanwezigheid van een gebande textuur.</v>
       </c>
       <c r="H18" t="str">
-        <v>null</v>
+        <v>geband</v>
       </c>
       <c r="I18" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J18" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/23</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/go</v>
       </c>
       <c r="B19" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C19" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.go</v>
       </c>
       <c r="D19" t="str">
-        <v>null</v>
+        <v>Een laagvlak dat een ondulerend of golvend voorkomen heeft, in tegenstelling tot een recht laagvlak.</v>
       </c>
       <c r="E19" t="str">
-        <v>packstone textuur</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F19" t="str">
-        <v>23</v>
+        <v>GO</v>
       </c>
       <c r="G19" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Een laagvlak dat een ondulerend of golvend voorkomen heeft, in tegenstelling tot een recht laagvlak.</v>
       </c>
       <c r="H19" t="str">
-        <v>null</v>
+        <v>golvend laagvlak</v>
       </c>
       <c r="I19" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J19" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/24</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/gp</v>
       </c>
       <c r="B20" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C20" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.gp</v>
       </c>
       <c r="D20" t="str">
-        <v>null</v>
+        <v>Structuur gevormd door de gedeeltelijke opvulling van een holte door sediment onder invloed van de zwaartekracht.</v>
       </c>
       <c r="E20" t="str">
-        <v>grainstone textuur</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F20" t="str">
-        <v>24</v>
+        <v>GP</v>
       </c>
       <c r="G20" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Structuur gevormd door de gedeeltelijke opvulling van een holte door sediment onder invloed van de zwaartekracht.</v>
       </c>
       <c r="H20" t="str">
-        <v>null</v>
+        <v>geopetale structuur</v>
       </c>
       <c r="I20" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J20" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/25</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/gt</v>
       </c>
       <c r="B21" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C21" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.gt</v>
       </c>
       <c r="D21" t="str">
-        <v>null</v>
+        <v>De textuur van een klastisch gesteente.</v>
       </c>
       <c r="E21" t="str">
-        <v>boundstone textuur</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F21" t="str">
-        <v>25</v>
+        <v>GT</v>
       </c>
       <c r="G21" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>De textuur van een klastisch gesteente.</v>
       </c>
       <c r="H21" t="str">
-        <v>null</v>
+        <v>grainstone textuur</v>
       </c>
       <c r="I21" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J21" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/26</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/hg</v>
       </c>
       <c r="B22" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C22" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.hg</v>
       </c>
       <c r="D22" t="str">
-        <v>null</v>
+        <v>Een verhard oppervlak, gevormd door synsedimentaire lithificatie van sediment op de zeebodem tijdens een periode van verminderde sedimentatiesnelheid.</v>
       </c>
       <c r="E22" t="str">
-        <v>karst / oplossing</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F22" t="str">
-        <v>26</v>
+        <v>HG</v>
       </c>
       <c r="G22" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Een verhard oppervlak, gevormd door synsedimentaire lithificatie van sediment op de zeebodem tijdens een periode van verminderde sedimentatiesnelheid.</v>
       </c>
       <c r="H22" t="str">
-        <v>null</v>
+        <v>hardground</v>
       </c>
       <c r="I22" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J22" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/27</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/ik</v>
       </c>
       <c r="B23" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C23" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.ik</v>
       </c>
       <c r="D23" t="str">
-        <v>null</v>
+        <v>Een klast gevormd door erosie van sediment niet lang na afzetting, herwerkt in een jongere afzetting.</v>
       </c>
       <c r="E23" t="str">
-        <v>hardground</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F23" t="str">
-        <v>27</v>
+        <v>IK</v>
       </c>
       <c r="G23" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Een klast gevormd door erosie van sediment niet lang na afzetting, herwerkt in een jongere afzetting.</v>
       </c>
       <c r="H23" t="str">
-        <v>null</v>
+        <v>intraklasten</v>
       </c>
       <c r="I23" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J23" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/28</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/ka</v>
       </c>
       <c r="B24" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C24" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.ka</v>
       </c>
       <c r="D24" t="str">
-        <v>null</v>
+        <v>Oplossingsstructuren gevormd in carbonaathoudend materiaal, meestal door de inwerking van zuur oppervlaktewater.</v>
       </c>
       <c r="E24" t="str">
-        <v>concretie</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F24" t="str">
-        <v>28</v>
+        <v>KA</v>
       </c>
       <c r="G24" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Oplossingsstructuren gevormd in carbonaathoudend materiaal, meestal door de inwerking van zuur oppervlaktewater.</v>
       </c>
       <c r="H24" t="str">
-        <v>null</v>
+        <v>karst / oplossing</v>
       </c>
       <c r="I24" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J24" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/29</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/ke</v>
       </c>
       <c r="B25" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C25" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.ke</v>
       </c>
       <c r="D25" t="str">
-        <v>null</v>
+        <v>Laagjes of discontinue lenzen van klei.</v>
       </c>
       <c r="E25" t="str">
-        <v>versteend / aaneengekit materiaal</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F25" t="str">
-        <v>29</v>
+        <v>KE</v>
       </c>
       <c r="G25" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Laagjes of discontinue lenzen van klei.</v>
       </c>
       <c r="H25" t="str">
-        <v>null</v>
+        <v>kleilenzen /-laagjes</v>
       </c>
       <c r="I25" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J25" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/3</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/kk</v>
       </c>
       <c r="B26" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C26" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.kk</v>
       </c>
       <c r="D26" t="str">
-        <v>null</v>
+        <v>Een klast bestaande uit kalkmateriaal.</v>
       </c>
       <c r="E26" t="str">
-        <v>geband</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F26" t="str">
-        <v>3</v>
+        <v>KK</v>
       </c>
       <c r="G26" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Een klast bestaande uit kalkmateriaal.</v>
       </c>
       <c r="H26" t="str">
-        <v>null</v>
+        <v>kalkklasten</v>
       </c>
       <c r="I26" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J26" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/30</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/kl</v>
       </c>
       <c r="B27" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C27" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.kl</v>
       </c>
       <c r="D27" t="str">
-        <v>null</v>
+        <v>Klasten bestaande uit kleiig materiaal.</v>
       </c>
       <c r="E27" t="str">
-        <v>uitdrogingsspleten</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F27" t="str">
-        <v>30</v>
+        <v>KL</v>
       </c>
       <c r="G27" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Klasten bestaande uit kleiig materiaal.</v>
       </c>
       <c r="H27" t="str">
-        <v>null</v>
+        <v>kleiklasten</v>
       </c>
       <c r="I27" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J27" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/31</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/ko</v>
       </c>
       <c r="B28" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C28" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.ko</v>
       </c>
       <c r="D28" t="str">
-        <v>null</v>
+        <v>Een laagvlak rijk aan brokjes van bruinkool of steenkool.</v>
       </c>
       <c r="E28" t="str">
-        <v>bioklasten</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F28" t="str">
-        <v>31</v>
+        <v>KO</v>
       </c>
       <c r="G28" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Een laagvlak rijk aan brokjes van bruinkool of steenkool.</v>
       </c>
       <c r="H28" t="str">
-        <v>null</v>
+        <v>laagvlak met koolbrokjes</v>
       </c>
       <c r="I28" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J28" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/32</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/kr</v>
       </c>
       <c r="B29" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C29" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.kr</v>
       </c>
       <c r="D29" t="str">
-        <v>null</v>
+        <v>Sedimentaire structuur waarbij schuine gelaagdheden voorkomen in verschillende tegengestelde oriëntaties.</v>
       </c>
       <c r="E29" t="str">
-        <v>pellets</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F29" t="str">
-        <v>32</v>
+        <v>KR</v>
       </c>
       <c r="G29" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Sedimentaire structuur waarbij schuine gelaagdheden voorkomen in verschillende tegengestelde oriëntaties.</v>
       </c>
       <c r="H29" t="str">
-        <v>null</v>
+        <v>kriskras gelaagdheid</v>
       </c>
       <c r="I29" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J29" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/33</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/kv</v>
       </c>
       <c r="B30" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C30" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.kv</v>
       </c>
       <c r="D30" t="str">
-        <v>null</v>
+        <v>Een laagvlak bestaande uit kleiig materiaal.</v>
       </c>
       <c r="E30" t="str">
-        <v>oölieten</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F30" t="str">
-        <v>33</v>
+        <v>KV</v>
       </c>
       <c r="G30" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Een laagvlak bestaande uit kleiig materiaal.</v>
       </c>
       <c r="H30" t="str">
-        <v>null</v>
+        <v>kleirijk laagvlak</v>
       </c>
       <c r="I30" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J30" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/34</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/la</v>
       </c>
       <c r="B31" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C31" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.la</v>
       </c>
       <c r="D31" t="str">
-        <v>null</v>
+        <v>Fijne discrete laagjes in het sediment of gesteente, tussen 0,005 en 1 mm dik.</v>
       </c>
       <c r="E31" t="str">
-        <v>oncolieten</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F31" t="str">
-        <v>34</v>
+        <v>LA</v>
       </c>
       <c r="G31" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Fijne discrete laagjes in het sediment of gesteente, tussen 0,005 en 1 mm dik.</v>
       </c>
       <c r="H31" t="str">
-        <v>null</v>
+        <v>laminaties</v>
       </c>
       <c r="I31" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J31" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/35</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/le</v>
       </c>
       <c r="B32" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C32" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.le</v>
       </c>
       <c r="D32" t="str">
-        <v>null</v>
+        <v>Voorkomen van lensvormige discontinue laagjes.</v>
       </c>
       <c r="E32" t="str">
-        <v>pisolieten</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F32" t="str">
-        <v>35</v>
+        <v>LE</v>
       </c>
       <c r="G32" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Voorkomen van lensvormige discontinue laagjes.</v>
       </c>
       <c r="H32" t="str">
-        <v>null</v>
+        <v>lensvormige gelaagdheid</v>
       </c>
       <c r="I32" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J32" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/36</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/lf</v>
       </c>
       <c r="B33" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C33" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.lf</v>
       </c>
       <c r="D33" t="str">
-        <v>null</v>
+        <v>Geëlongeerde dunne holten in sedimentaire gesteenten, geheel of gedeeltelijk opgevuld.</v>
       </c>
       <c r="E33" t="str">
-        <v>intraklasten</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F33" t="str">
-        <v>36</v>
+        <v>LF</v>
       </c>
       <c r="G33" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Geëlongeerde dunne holten in sedimentaire gesteenten, geheel of gedeeltelijk opgevuld.</v>
       </c>
       <c r="H33" t="str">
-        <v>null</v>
+        <v>laminoid-fenestral structuur</v>
       </c>
       <c r="I33" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J33" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/37</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/li</v>
       </c>
       <c r="B34" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C34" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.li</v>
       </c>
       <c r="D34" t="str">
-        <v>null</v>
+        <v>Banken bestaande uit ligniet of bruinkool.</v>
       </c>
       <c r="E34" t="str">
-        <v>evaporiet pseudomorfen</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F34" t="str">
-        <v>37</v>
+        <v>LI</v>
       </c>
       <c r="G34" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Banken bestaande uit ligniet of bruinkool.</v>
       </c>
       <c r="H34" t="str">
-        <v>null</v>
+        <v>lignietbanken</v>
       </c>
       <c r="I34" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J34" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/38</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/lm</v>
       </c>
       <c r="B35" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C35" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.lm</v>
       </c>
       <c r="D35" t="str">
-        <v>null</v>
+        <v>Banken die verhard zijn door de oxidatie van ijzerhoudende mineralen en de vorming van limoniet.</v>
       </c>
       <c r="E35" t="str">
-        <v>calcrete / caliche</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F35" t="str">
-        <v>38</v>
+        <v>LM</v>
       </c>
       <c r="G35" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Banken die verhard zijn door de oxidatie van ijzerhoudende mineralen en de vorming van limoniet.</v>
       </c>
       <c r="H35" t="str">
-        <v>null</v>
+        <v>limoniet- / ijzerbanken</v>
       </c>
       <c r="I35" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J35" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/4</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/lo</v>
       </c>
       <c r="B36" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C36" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.lo</v>
       </c>
       <c r="D36" t="str">
-        <v>null</v>
+        <v>Structuur gevormd bij deformatie van nat sediment, bv. nadat zand wordt afgezet bovenop klei waarbij het zand deels inzakt en ronde afdrukken achterlaat in de klei.</v>
       </c>
       <c r="E36" t="str">
-        <v>lensvormige gelaagdheid</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F36" t="str">
-        <v>4</v>
+        <v>LO</v>
       </c>
       <c r="G36" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Structuur gevormd bij deformatie van nat sediment, bv. nadat zand wordt afgezet bovenop klei waarbij het zand deels inzakt en ronde afdrukken achterlaat in de klei.</v>
       </c>
       <c r="H36" t="str">
-        <v>null</v>
+        <v>load cast</v>
       </c>
       <c r="I36" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J36" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/40</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/ma</v>
       </c>
       <c r="B37" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C37" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.ma</v>
       </c>
       <c r="D37" t="str">
-        <v>null</v>
+        <v>Zonder interne structuur.</v>
       </c>
       <c r="E37" t="str">
-        <v>FU-gegradeerde gelaagdheid</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F37" t="str">
-        <v>40</v>
+        <v>MA</v>
       </c>
       <c r="G37" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Zonder interne structuur.</v>
       </c>
       <c r="H37" t="str">
-        <v>null</v>
+        <v>massief (compact)</v>
       </c>
       <c r="I37" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J37" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/41</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/mi</v>
       </c>
       <c r="B38" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C38" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.mi</v>
       </c>
       <c r="D38" t="str">
-        <v>null</v>
+        <v>Een vlak rijk aan mica's of glimmers, plaatvormige fyllosilicaten.</v>
       </c>
       <c r="E38" t="str">
-        <v>CU-gegradeerde gelaagdheid</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F38" t="str">
-        <v>41</v>
+        <v>MI</v>
       </c>
       <c r="G38" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Een vlak rijk aan mica's of glimmers, plaatvormige fyllosilicaten.</v>
       </c>
       <c r="H38" t="str">
-        <v>null</v>
+        <v>micarijk vlak</v>
       </c>
       <c r="I38" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J38" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/42</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/mu</v>
       </c>
       <c r="B39" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C39" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.mu</v>
       </c>
       <c r="D39" t="str">
-        <v>null</v>
+        <v>Gesteente met een zeer fijne kleiige textuur.</v>
       </c>
       <c r="E39" t="str">
-        <v>turbidiet</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F39" t="str">
-        <v>42</v>
+        <v>MU</v>
       </c>
       <c r="G39" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Gesteente met een zeer fijne kleiige textuur.</v>
       </c>
       <c r="H39" t="str">
-        <v>null</v>
+        <v>mudstone textuur</v>
       </c>
       <c r="I39" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J39" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/43</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/no</v>
       </c>
       <c r="B40" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C40" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.no</v>
       </c>
       <c r="D40" t="str">
-        <v>null</v>
+        <v>Een sedimentair gesteente rijk aan afgeronde vormen (nodules).</v>
       </c>
       <c r="E40" t="str">
-        <v>speleotheem</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F40" t="str">
-        <v>43</v>
+        <v>NO</v>
       </c>
       <c r="G40" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Een sedimentair gesteente rijk aan afgeronde vormen (nodules).</v>
       </c>
       <c r="H40" t="str">
-        <v>null</v>
+        <v>nodulair</v>
       </c>
       <c r="I40" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J40" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/44</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/ob</v>
       </c>
       <c r="B41" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C41" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.ob</v>
       </c>
       <c r="D41" t="str">
-        <v>null</v>
+        <v>Sedimentaire structuur onbepaald</v>
       </c>
       <c r="E41" t="str">
-        <v>birdseyes</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F41" t="str">
-        <v>44</v>
+        <v>OB</v>
       </c>
       <c r="G41" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Sedimentaire structuur onbepaald</v>
       </c>
       <c r="H41" t="str">
-        <v>null</v>
+        <v>onbepaald</v>
       </c>
       <c r="I41" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J41" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/45</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/on</v>
       </c>
       <c r="B42" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C42" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.on</v>
       </c>
       <c r="D42" t="str">
-        <v>null</v>
+        <v>Een korrel met carbonaatcoating gevormd door microbiële matten met irregulaire laminae.</v>
       </c>
       <c r="E42" t="str">
-        <v>stroomribbels</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F42" t="str">
-        <v>45</v>
+        <v>ON</v>
       </c>
       <c r="G42" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Een korrel met carbonaatcoating gevormd door microbiële matten met irregulaire laminae.</v>
       </c>
       <c r="H42" t="str">
-        <v>null</v>
+        <v>oncolieten</v>
       </c>
       <c r="I42" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J42" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/46</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/oo</v>
       </c>
       <c r="B43" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C43" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.oo</v>
       </c>
       <c r="D43" t="str">
-        <v>null</v>
+        <v>Een kleine (&lt; 2 mm) korrel met carbonaat- of ijzercoating met een cortex van fijne concentrische laminae zonder biogene eigenschappen en een nucleus bestaande uit een schelpfragment of een zandkorrel.</v>
       </c>
       <c r="E43" t="str">
-        <v>fijn gebankt</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F43" t="str">
-        <v>46</v>
+        <v>OO</v>
       </c>
       <c r="G43" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Een kleine (&lt; 2 mm) korrel met carbonaat- of ijzercoating met een cortex van fijne concentrische laminae zonder biogene eigenschappen en een nucleus bestaande uit een schelpfragment of een zandkorrel.</v>
       </c>
       <c r="H43" t="str">
-        <v>null</v>
+        <v>oölieten</v>
       </c>
       <c r="I43" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J43" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/47</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/pe</v>
       </c>
       <c r="B44" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C44" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.pe</v>
       </c>
       <c r="D44" t="str">
-        <v>null</v>
+        <v>Een ovoïde tot sferisch micriet deeltje zonder interne structuur, met een diameter van 0,03 tot 0,15 mm.</v>
       </c>
       <c r="E44" t="str">
-        <v>kleiklasten</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F44" t="str">
-        <v>47</v>
+        <v>PE</v>
       </c>
       <c r="G44" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Een ovoïde tot sferisch micriet deeltje zonder interne structuur, met een diameter van 0,03 tot 0,15 mm.</v>
       </c>
       <c r="H44" t="str">
-        <v>null</v>
+        <v>pellets</v>
       </c>
       <c r="I44" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J44" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/48</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/pi</v>
       </c>
       <c r="B45" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C45" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.pi</v>
       </c>
       <c r="D45" t="str">
-        <v>null</v>
+        <v>Een korrel met carbonaatcoating groter dan 2 mm in diameter.</v>
       </c>
       <c r="E45" t="str">
-        <v>golvend laagvlak</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F45" t="str">
-        <v>48</v>
+        <v>PI</v>
       </c>
       <c r="G45" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Een korrel met carbonaatcoating groter dan 2 mm in diameter.</v>
       </c>
       <c r="H45" t="str">
-        <v>null</v>
+        <v>pisoiden</v>
       </c>
       <c r="I45" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J45" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/49</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/pl</v>
       </c>
       <c r="B46" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C46" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.pl</v>
       </c>
       <c r="D46" t="str">
-        <v>null</v>
+        <v>Mengsel van plantenresten.</v>
       </c>
       <c r="E46" t="str">
-        <v>breccieus</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F46" t="str">
-        <v>49</v>
+        <v>PL</v>
       </c>
       <c r="G46" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Mengsel van plantenresten.</v>
       </c>
       <c r="H46" t="str">
-        <v>null</v>
+        <v>aangespoelde plantenresten / plantenhaksel</v>
       </c>
       <c r="I46" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J46" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/5</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/ps</v>
       </c>
       <c r="B47" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C47" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.ps</v>
       </c>
       <c r="D47" t="str">
-        <v>null</v>
+        <v>Een gesteente bestaande uit pisoiden.</v>
       </c>
       <c r="E47" t="str">
-        <v>massief (compact)</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F47" t="str">
-        <v>5</v>
+        <v>PS</v>
       </c>
       <c r="G47" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Een gesteente bestaande uit pisoiden.</v>
       </c>
       <c r="H47" t="str">
-        <v>null</v>
+        <v>pisolieten</v>
       </c>
       <c r="I47" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J47" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/50</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/pt</v>
       </c>
       <c r="B48" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C48" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.pt</v>
       </c>
       <c r="D48" t="str">
-        <v>null</v>
+        <v>Klastische kalksteen waarbij de korrels elkaar ondersteunen, met een beperkte hoeveelheid kalkmodder.</v>
       </c>
       <c r="E48" t="str">
-        <v>kleilenzen /-laagjes</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F48" t="str">
-        <v>50</v>
+        <v>PT</v>
       </c>
       <c r="G48" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Klastische kalksteen waarbij de korrels elkaar ondersteunen, met een beperkte hoeveelheid kalkmodder.</v>
       </c>
       <c r="H48" t="str">
-        <v>null</v>
+        <v>packstone textuur</v>
       </c>
       <c r="I48" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J48" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/51</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/re</v>
       </c>
       <c r="B49" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C49" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.re</v>
       </c>
       <c r="D49" t="str">
-        <v>null</v>
+        <v>Cilindrische vormen en afdrukken in het gesteente, bv. door graafactiviteit van organismen.</v>
       </c>
       <c r="E49" t="str">
-        <v>kalkklasten</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F49" t="str">
-        <v>51</v>
+        <v>RE</v>
       </c>
       <c r="G49" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Cilindrische vormen en afdrukken in het gesteente, bv. door graafactiviteit van organismen.</v>
       </c>
       <c r="H49" t="str">
-        <v>null</v>
+        <v>'regendruppels' (cf. Planolites)</v>
       </c>
       <c r="I49" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J49" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/52</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/ru</v>
       </c>
       <c r="B50" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C50" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.ru</v>
       </c>
       <c r="D50" t="str">
-        <v>null</v>
+        <v>Een klastisch gesteente met meer dan 30 % grindkorrels (&gt; 2 mm), met of zonder een matrix van zand en/of klei.</v>
       </c>
       <c r="E50" t="str">
-        <v>fossielrijk</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F50" t="str">
-        <v>52</v>
+        <v>RU</v>
       </c>
       <c r="G50" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Een klastisch gesteente met meer dan 30 % grindkorrels (&gt; 2 mm), met of zonder een matrix van zand en/of klei.</v>
       </c>
       <c r="H50" t="str">
-        <v>null</v>
+        <v>rudstone</v>
       </c>
       <c r="I50" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J50" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/53</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/sg</v>
       </c>
       <c r="B51" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C51" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.sg</v>
       </c>
       <c r="D51" t="str">
-        <v>null</v>
+        <v>De karakteristieke structuur gevormd door de stroomafwaartse migratie van onderwaterstructuren met een schuin sedimentair oppervlak.</v>
       </c>
       <c r="E51" t="str">
-        <v>nodulair</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F51" t="str">
-        <v>53</v>
+        <v>SG</v>
       </c>
       <c r="G51" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>De karakteristieke structuur gevormd door de stroomafwaartse migratie van onderwaterstructuren met een schuin sedimentair oppervlak.</v>
       </c>
       <c r="H51" t="str">
-        <v>null</v>
+        <v>schuine gelaagdheid</v>
       </c>
       <c r="I51" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J51" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/54</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/sl</v>
       </c>
       <c r="B52" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C52" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.sl</v>
       </c>
       <c r="D52" t="str">
-        <v>null</v>
+        <v>Neerwaarts massatransport van sediment onder invloed van de zwaartekracht. Vaak sterke interne deformatie.</v>
       </c>
       <c r="E52" t="str">
-        <v>kleirijk laagvlak</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F52" t="str">
-        <v>54</v>
+        <v>SL</v>
       </c>
       <c r="G52" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Neerwaarts massatransport van sediment onder invloed van de zwaartekracht. Vaak sterke interne deformatie.</v>
       </c>
       <c r="H52" t="str">
-        <v>null</v>
+        <v>slumping</v>
       </c>
       <c r="I52" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J52" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/55</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/sp</v>
       </c>
       <c r="B53" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C53" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.sp</v>
       </c>
       <c r="D53" t="str">
-        <v>null</v>
+        <v>Een chemische neerslag gevormd in een grot (bv. stalagmieten en stalactieten). Doorgaans bestaande uit calciet, maar soms ook gips of haliet.</v>
       </c>
       <c r="E53" t="str">
-        <v>floatstone</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F53" t="str">
-        <v>55</v>
+        <v>SP</v>
       </c>
       <c r="G53" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Een chemische neerslag gevormd in een grot (bv. stalagmieten en stalactieten). Doorgaans bestaande uit calciet, maar soms ook gips of haliet.</v>
       </c>
       <c r="H53" t="str">
-        <v>null</v>
+        <v>speleotheem</v>
       </c>
       <c r="I53" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J53" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/56</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/sr</v>
       </c>
       <c r="B54" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C54" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.sr</v>
       </c>
       <c r="D54" t="str">
-        <v>null</v>
+        <v>Golvende structuren of ribbels gevormd door de stroming van water.</v>
       </c>
       <c r="E54" t="str">
-        <v>rudstone</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F54" t="str">
-        <v>56</v>
+        <v>SR</v>
       </c>
       <c r="G54" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Golvende structuren of ribbels gevormd door de stroming van water.</v>
       </c>
       <c r="H54" t="str">
-        <v>null</v>
+        <v>stroomribbels</v>
       </c>
       <c r="I54" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J54" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/57</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/st</v>
       </c>
       <c r="B55" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C55" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.st</v>
       </c>
       <c r="D55" t="str">
-        <v>null</v>
+        <v>Afzetting, sediment of gesteente met duidelijk herkenbare gelaagdheid of stratificatie.</v>
       </c>
       <c r="E55" t="str">
-        <v>pisoiden</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F55" t="str">
-        <v>57</v>
+        <v>ST</v>
       </c>
       <c r="G55" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Afzetting, sediment of gesteente met duidelijk herkenbare gelaagdheid of stratificatie.</v>
       </c>
       <c r="H55" t="str">
-        <v>null</v>
+        <v>stratificaties</v>
       </c>
       <c r="I55" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J55" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/58</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/tu</v>
       </c>
       <c r="B56" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C56" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.tu</v>
       </c>
       <c r="D56" t="str">
-        <v>null</v>
+        <v>Een afzetting gevormd onder invloed van een onderwater densiteitsstroming van sediment in suspensie, onder invloed van de zwaartekracht, met het potentieel om over zeer zachte hellingen (&lt; 1%) naar beneden of zelfs hellingopwaarts te stromen.</v>
       </c>
       <c r="E56" t="str">
-        <v>laminoid-fenestral structuur</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F56" t="str">
-        <v>58</v>
+        <v>TU</v>
       </c>
       <c r="G56" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Een afzetting gevormd onder invloed van een onderwater densiteitsstroming van sediment in suspensie, onder invloed van de zwaartekracht, met het potentieel om over zeer zachte hellingen (&lt; 1%) naar beneden of zelfs hellingopwaarts te stromen.</v>
       </c>
       <c r="H56" t="str">
-        <v>null</v>
+        <v>turbidiet</v>
       </c>
       <c r="I56" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J56" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/59</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/us</v>
       </c>
       <c r="B57" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C57" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.us</v>
       </c>
       <c r="D57" t="str">
-        <v>null</v>
+        <v>Spleten gevormd door uitdroging, vaak in hexagonaal patroon en gevormd in kleiig sediment.</v>
       </c>
       <c r="E57" t="str">
-        <v>limoniet- / ijzerbanken</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F57" t="str">
-        <v>59</v>
+        <v>US</v>
       </c>
       <c r="G57" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Spleten gevormd door uitdroging, vaak in hexagonaal patroon en gevormd in kleiig sediment.</v>
       </c>
       <c r="H57" t="str">
-        <v>null</v>
+        <v>uitdrogingsspleten</v>
       </c>
       <c r="I57" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J57" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/6</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/vb</v>
       </c>
       <c r="B58" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C58" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.vb</v>
       </c>
       <c r="D58" t="str">
-        <v>null</v>
+        <v>Banken bestaande uit veen of turf, afgestorven en zeer licht gecompacteerd organisch materiaal.</v>
       </c>
       <c r="E58" t="str">
-        <v>zandwolken</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F58" t="str">
-        <v>6</v>
+        <v>VB</v>
       </c>
       <c r="G58" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Banken bestaande uit veen of turf, afgestorven en zeer licht gecompacteerd organisch materiaal.</v>
       </c>
       <c r="H58" t="str">
-        <v>null</v>
+        <v>veenbanken</v>
       </c>
       <c r="I58" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J58" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/60</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/vk</v>
       </c>
       <c r="B59" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C59" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.vk</v>
       </c>
       <c r="D59" t="str">
-        <v>null</v>
+        <v>Verspreid voorkomen van keien of grind (&gt; 2 mm).</v>
       </c>
       <c r="E59" t="str">
-        <v>lignietbanken</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F59" t="str">
-        <v>60</v>
+        <v>VK</v>
       </c>
       <c r="G59" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Verspreid voorkomen van keien of grind (&gt; 2 mm).</v>
       </c>
       <c r="H59" t="str">
-        <v>null</v>
+        <v>verspreide keien</v>
       </c>
       <c r="I59" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J59" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/61</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/vs</v>
       </c>
       <c r="B60" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C60" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.vs</v>
       </c>
       <c r="D60" t="str">
-        <v>null</v>
+        <v>Materiaal dat (deels) versteend of aaneengekit is, bv. door een cement van kalk, ijzeroxiden of silica.</v>
       </c>
       <c r="E60" t="str">
-        <v>veenbanken</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F60" t="str">
-        <v>61</v>
+        <v>VS</v>
       </c>
       <c r="G60" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Materiaal dat (deels) versteend of aaneengekit is, bv. door een cement van kalk, ijzeroxiden of silica.</v>
       </c>
       <c r="H60" t="str">
-        <v>null</v>
+        <v>versteend / aaneengekit materiaal</v>
       </c>
       <c r="I60" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J60" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/62</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/wa</v>
       </c>
       <c r="B61" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C61" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.wa</v>
       </c>
       <c r="D61" t="str">
-        <v>null</v>
+        <v>Een kalksteen met carbonaatdeeltjes die worden ondersteund door een matrix van fijne kalkmodder.</v>
       </c>
       <c r="E61" t="str">
-        <v>geopetale structuur</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F61" t="str">
-        <v>62</v>
+        <v>WA</v>
       </c>
       <c r="G61" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Een kalksteen met carbonaatdeeltjes die worden ondersteund door een matrix van fijne kalkmodder.</v>
       </c>
       <c r="H61" t="str">
-        <v>null</v>
+        <v>wackestone textuur</v>
       </c>
       <c r="I61" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J61" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/7</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/zk</v>
       </c>
       <c r="B62" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C62" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.zk</v>
       </c>
       <c r="D62" t="str">
-        <v>null</v>
+        <v>Een laagvlak met een zwarte kleur door verhoogd organisch materiaal.</v>
       </c>
       <c r="E62" t="str">
-        <v>schuine gelaagdheid</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F62" t="str">
-        <v>7</v>
+        <v>ZK</v>
       </c>
       <c r="G62" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Een laagvlak met een zwarte kleur door verhoogd organisch materiaal.</v>
       </c>
       <c r="H62" t="str">
-        <v>null</v>
+        <v>zwart / kolig laagvlak</v>
       </c>
       <c r="I62" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J62" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/8</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/zw</v>
       </c>
       <c r="B63" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C63" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.sedimentairestructuurtype.zw</v>
       </c>
       <c r="D63" t="str">
-        <v>null</v>
+        <v>Lokaal voorkomen van een zandconcentratie in een ander materiaal.</v>
       </c>
       <c r="E63" t="str">
-        <v>kriskras gelaagdheid</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="F63" t="str">
-        <v>8</v>
+        <v>ZW</v>
       </c>
       <c r="G63" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>Lokaal voorkomen van een zandconcentratie in een ander materiaal.</v>
       </c>
       <c r="H63" t="str">
-        <v>null</v>
+        <v>zandwolken</v>
       </c>
       <c r="I63" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+      </c>
+      <c r="J63" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/9</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
       </c>
       <c r="B64" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
+        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
       </c>
       <c r="C64" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.conceptscheme.sedimentairestructuurtype</v>
       </c>
       <c r="D64" t="str">
         <v>null</v>
       </c>
       <c r="E64" t="str">
-        <v>load cast</v>
+        <v>null</v>
       </c>
       <c r="F64" t="str">
-        <v>9</v>
+        <v>null</v>
       </c>
       <c r="G64" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
+        <v>null</v>
       </c>
       <c r="H64" t="str">
-        <v>null</v>
+        <v>Lijst van types sedimentaire structuren</v>
       </c>
       <c r="I64" t="str">
         <v>null</v>
       </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/sedimentairestructuurtype</v>
-      </c>
-      <c r="B65" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
-      </c>
-      <c r="C65" t="str">
-        <v>null</v>
-      </c>
-      <c r="D65" t="str">
-        <v>null</v>
-      </c>
-      <c r="E65" t="str">
-        <v>Lijst van types sedimentaire structuren</v>
-      </c>
-      <c r="F65" t="str">
-        <v>null</v>
-      </c>
-      <c r="G65" t="str">
-        <v>null</v>
-      </c>
-      <c r="H65" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.conceptscheme.sedimentairestructuurtype</v>
-      </c>
-      <c r="I65" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/0|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/10|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/11|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/12|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/13|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/14|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/15|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/16|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/17|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/18|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/19|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/1|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/20|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/21|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/22|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/23|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/24|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/25|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/26|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/27|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/28|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/29|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/2|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/30|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/31|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/32|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/33|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/34|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/35|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/36|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/37|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/38|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/3|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/40|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/41|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/42|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/43|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/44|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/45|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/46|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/47|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/48|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/49|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/4|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/50|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/51|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/52|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/53|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/54|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/55|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/56|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/57|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/58|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/59|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/5|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/60|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/61|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/62|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/6|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/7|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/8|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/9</v>
+      <c r="J64" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/be|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/bk|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/bo|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/br|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/bt|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/ca|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/cb|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/co|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/cu|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/ep|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/ev|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/fb|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/fn|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/fo|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/fs|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/fu|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/ge|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/go|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/gp|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/gt|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/hg|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/ik|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/ka|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/ke|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/kk|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/kl|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/ko|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/kr|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/kv|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/la|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/le|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/lf|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/li|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/lm|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/lo|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/ma|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/mi|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/mu|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/no|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/ob|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/on|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/oo|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/pe|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/pi|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/pl|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/ps|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/pt|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/re|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/ru|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/sg|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/sl|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/sp|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/sr|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/st|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/tu|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/us|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/vb|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/vk|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/vs|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/wa|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/zk|https://data.bodemenondergrond.vlaanderen.be/id/concept/sedimentairestructuurtype/zw</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I65"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J64"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>